<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-04 La cabane sous la table
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-04.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-04.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, sous la table, nappe savon, après le déjeuner</t>
+          <t>salon après le déjeuner, nappe savon, dessous de table, caisse bleue</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut une cabane sous la table, avec son doudou. Les voitures bleues recouvrent le doudou. Elle les met dans la caisse pour voir dessous. Le doudou apparaît. La cabane est douce.</t>
+          <t>Le torchon glisse. Une cuillère tinte. Au pied de la chaise, un éclat d'ombre brille. Sarah veut sa cabane sous la table, maintenant. Elle pousse le coussin d'un coup : une voiture touche son genou, le doudou disparaît. Première idée ratée. Elle refuse de foncer, pose les voitures dans la caisse. L'éclat d'ombre montre le rose. Merci vécu. Au plafond de nappe, l'éclat d'ombre dore.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une ombre de chaise coupe le tapis. L'ombre est longue, un peu froide. La nappe sent encore le savon. Une cuillère tinte, loin, dans un verre. J'essuie la table, Sarah. Je prends un coussin. Sous la table, il fait sombre. C'est calme, tout petit. En ce moment, Sarah glisse dessous. Ses genoux trouvent le tapis. Des voitures bleues attendent. Elles sont lisses, un peu froides. Elles roulent, papa. Elles roulent dans l'ombre. Sarah pousse une voiture. Vroom. Puis une autre. Vroom. Elle aligne trois voitures bleues. Elles se touchent, tout doucement. C'est un parking ? Oui, sous la table. Le doudou rose est près d'elle. Toi, tu restes dans la cabane. Sarah le pose contre un pied. Une voiture glisse vers lui. Puis une autre. Les voitures le recouvrent un peu. Après, c'est ma cabane. Avec le coussin ? Oui, une cabane. Maman tend le coussin. Il est moelleux. Sarah veut le glisser dessous. Une voiture touche son genou. Aïe. La voiture est là. Où est mon doudou ? Sur la chaise, peut-être ? Sarah sort la tête. La chaise est vide. Dans le coussin ? Elle fouille le tissu. Rien. Il est perdu. Les voitures sont encore au sol. Je veux voir dessous. Sarah prend une voiture bleue. Elle la pose dans la caisse bleue. Clac.</t>
+          <t>Le torchon glisse sur le bois. Ça sent le savon, tiède. J'essuie la table, Sarah. Une cuillère tinte dans un verre. Au pied de la chaise, un éclat d'ombre brille. Il est petit, papa. C'est l'ombre de la chaise. L'éclat d'ombre coupe le tapis. La nappe sent le savon. Un coin de nappe tombe vers le tapis. Je prends le coussin. Sous la table, il fait sombre. Sarah connaît ce dessous de table. Un détail paraît nouveau, là. L'éclat tremble sur le pied. En ce moment, Sarah glisse dessous. Je veux ma cabane, maintenant. Maintenant ? Oui, tout de suite. Tu la veux sous la table ? Oui, avec le coussin. Ses genoux trouvent le tapis. Le tapis est un peu froid. Des voitures bleues attendent. Elles sont lisses, un peu froides. Elles roulent, papa. Elles roulent dans l'ombre. Sarah pousse une voiture. Vroom. Puis une autre. Vroom. Elle aligne trois voitures bleues. Les roues sont froides sous le doigt. C'est un parking ? Oui, sous la table. Le doudou rose est près d'elle. Toi, tu restes dans la cabane. Sarah le pose contre un pied. Une voiture glisse vers lui. Une deuxième le recouvre. Le rose disparaît sous le bleu. Après, c'est ma cabane. Avec le coussin ? Oui, une cabane. Maman tend le coussin. Il est moelleux, un peu lourd. Sarah veut le glisser dessous. Elle pousse fort, d'un coup. Une voiture touche son genou. Aïe. La voiture est là. Le sourire de Sarah disparaît. Ses épaules tombent un peu. Où est mon doudou ? Sur la chaise, peut-être ? Sarah sort la tête. La chaise est vide. Dans le coussin ? Elle fouille le tissu. Rien. Il est perdu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes sous les voitures ? Je veux voir dessous. Sarah prend une voiture bleue. Elle la pose dans la caisse. Clac.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une ombre de chaise coupe le tapis. L'ombre est longue, un peu froide. La nappe sent encore le savon. Une cuillère tinte, loin, dans un verre. J'essuie la table, Sarah. Je prends un coussin. Sous la table, il fait sombre. C'est calme, tout petit. En ce moment, Sarah glisse dessous. Ses genoux trouvent le tapis. Des voitures bleues attendent. Elles sont lisses, un peu froides. Elles roulent, papa. Elles roulent dans l'ombre. Sarah pousse une voiture. Vroom. Puis une autre. Vroom. Elle aligne trois voitures bleues. Elles se touchent, tout doucement. C'est un parking ? Oui, sous la table. Le doudou rose est près d'elle. Toi, tu restes dans la cabane. Sarah le pose contre un pied. Une voiture glisse vers lui. Puis une autre. Les voitures le recouvrent un peu. Après, c'est ma cabane. Avec le coussin ? Oui, une cabane. Maman tend le coussin. Il est moelleux. Sarah veut le glisser dessous. Une voiture touche son genou. Aïe. La voiture est là. Où est mon doudou ? Sur la chaise, peut-être ? Sarah sort la tête. La chaise est vide. Dans le coussin ? Elle fouille le tissu. Rien. Il est perdu. Les voitures sont encore au sol. Je veux voir dessous. Sarah prend une voiture bleue. Elle la pose dans la caisse bleue. Clac.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le torchon glisse sur le bois. Ça sent le savon, tiède. J'essuie la table, Sarah. Une cuillère tinte dans un verre. Au pied de la chaise, un &lt;emphasis level="moderate"&gt;éclat d'ombre&lt;/emphasis&gt; brille. Il est petit, papa. C'est l'ombre de la chaise. L'éclat d'ombre coupe le tapis. La nappe sent le savon. Un coin de nappe tombe vers le tapis. Je prends le coussin. Sous la table, il fait sombre. Sarah connaît ce dessous de table. Un détail paraît nouveau, là. L'éclat tremble sur le pied. En ce moment, Sarah glisse dessous. Je veux ma cabane, maintenant. Maintenant ? Oui, tout de suite. Tu la veux sous la table ? Oui, avec le coussin. Ses genoux trouvent le tapis. Le tapis est un peu froid. Des voitures bleues attendent. Elles sont lisses, un peu froides. Elles roulent, papa. Elles roulent dans l'ombre. Sarah pousse une voiture. Vroom. Puis une autre. Vroom. Elle aligne trois voitures bleues. Les roues sont froides sous le doigt. C'est un parking ? Oui, sous la table. Le doudou rose est près d'elle. Toi, tu restes dans la cabane. Sarah le pose contre un pied. Une voiture glisse vers lui. Une deuxième le recouvre. Le rose disparaît sous le bleu. Après, c'est ma cabane. Avec le coussin ? Oui, une cabane. Maman tend le coussin. Il est moelleux, un peu lourd. Sarah veut le glisser dessous. Elle pousse fort, d'un coup. Une voiture touche son genou. Aïe. La voiture est là. Le sourire de Sarah disparaît. Ses épaules tombent un peu. Où est mon doudou ? Sur la chaise, peut-être ? Sarah sort la tête. La chaise est vide. Dans le coussin ? Elle fouille le tissu. Rien. Il est perdu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes sous les voitures ? Je veux voir dessous. Sarah prend une voiture bleue. Elle la pose dans la caisse. Clac.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Kenza a joué avec les voitures. Les voitures sont au sol. Papa dit : on range. Après le jeu, on range. Papa montre la caisse. La caisse est bleue. Kenza prend une voiture. Elle la met dans la caisse. Clac. Elle en prend une autre. Dans la caisse. Papa dit : les jouets retournent dans la caisse. Kenza répète : &lt;emphasis&gt;ranger&lt;/emphasis&gt;. Caisse. Elle met encore une voiture. La caisse se remplit. Le tapis est libre. Papa sourit. Kenza pousse la caisse. Elle est un peu lourde. Papa aide. Ils posent la caisse près du meuble. Kenza a rangé.&lt;/slow&gt; [pause]</t>
+          <t>Le torchon glisse sur le bois. Ça sent le savon, tiède. J'essuie la table, Sarah. Une cuillère tinte dans un verre. Au pied de la chaise, un &lt;emphasis&gt;éclat d'ombre&lt;/emphasis&gt; brille. Il est petit, papa. C'est l'ombre de la chaise. L'éclat d'ombre coupe le tapis. La nappe sent le savon. Un coin de nappe tombe vers le tapis. Je prends le coussin. Sous la table, il fait sombre. Sarah connaît ce dessous de table. Un détail paraît nouveau, là. L'éclat tremble sur le pied. En ce moment, Sarah glisse dessous. Je veux ma cabane, maintenant. Maintenant ? Oui, tout de suite. Tu la veux sous la table ? Oui, avec le coussin. Ses genoux trouvent le tapis. Le tapis est un peu froid. Des voitures bleues attendent. Elles sont lisses, un peu froides. Elles roulent, papa. Elles roulent dans l'ombre. Sarah pousse une voiture. Vroom. Puis une autre. Vroom. Elle aligne trois voitures bleues. Les roues sont froides sous le doigt. C'est un parking ? Oui, sous la table. Le doudou rose est près d'elle. Toi, tu restes dans la cabane. Sarah le pose contre un pied. Une voiture glisse vers lui. Une deuxième le recouvre. Le rose disparaît sous le bleu. Après, c'est ma cabane. Avec le coussin ? Oui, une cabane. Maman tend le coussin. Il est moelleux, un peu lourd. Sarah veut le glisser dessous. Elle pousse fort, d'un coup. Une voiture touche son genou. Aïe. La voiture est là. Le sourire de Sarah disparaît. Ses épaules tombent un peu. Où est mon doudou ? Sur la chaise, peut-être ? Sarah sort la tête. La chaise est vide. Dans le coussin ? Elle fouille le tissu. Rien. Il est perdu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes sous les voitures ? Je veux voir dessous. Sarah prend une voiture bleue. Elle la pose dans la caisse. Clac. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>éclat d'ombre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,21 +1319,38 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_cabane_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une ombre de chaise coupe le tapis.
-narrateur|L'ombre est longue, un peu froide.
-narrateur|La nappe sent encore le savon.
-narrateur|Une cuillère tinte, loin, dans un verre.
+          <t>narrateur|Le torchon glisse sur le bois.
+narrateur|Ça sent le savon, tiède.
 papa|J'essuie la table, Sarah.
-maman|Je prends un coussin.
+narrateur|Une cuillère tinte dans un verre.
+narrateur|Au pied de la chaise, un éclat d'ombre brille.
+enfant-f|Il est petit, papa.
+papa|C'est l'ombre de la chaise.
+narrateur|L'éclat d'ombre coupe le tapis.
+narrateur|La nappe sent le savon.
+narrateur|Un coin de nappe tombe vers le tapis.
+maman|Je prends le coussin.
 narrateur|Sous la table, il fait sombre.
-narrateur|C'est calme, tout petit.
+narrateur|Sarah connaît ce dessous de table.
+narrateur|Un détail paraît nouveau, là.
+narrateur|L'éclat tremble sur le pied.
 narrateur|En ce moment, Sarah glisse dessous.
+enfant-f|Je veux ma cabane, maintenant.
+papa|Maintenant ?
+enfant-f|Oui, tout de suite.
+maman|Tu la veux sous la table ?
+enfant-f|Oui, avec le coussin.
 narrateur|Ses genoux trouvent le tapis.
+narrateur|Le tapis est un peu froid.
 narrateur|Des voitures bleues attendent.
 narrateur|Elles sont lisses, un peu froides.
 enfant-f|Elles roulent, papa.
@@ -1343,24 +1360,27 @@
 narrateur|Puis une autre.
 narrateur|Vroom.
 narrateur|Elle aligne trois voitures bleues.
-narrateur|Elles se touchent, tout doucement.
+narrateur|Les roues sont froides sous le doigt.
 maman|C'est un parking ?
 enfant-f|Oui, sous la table.
 narrateur|Le doudou rose est près d'elle.
 enfant-f|Toi, tu restes dans la cabane.
 narrateur|Sarah le pose contre un pied.
 narrateur|Une voiture glisse vers lui.
-narrateur|Puis une autre.
-narrateur|Les voitures le recouvrent un peu.
+narrateur|Une deuxième le recouvre.
+narrateur|Le rose disparaît sous le bleu.
 enfant-f|Après, c'est ma cabane.
 maman|Avec le coussin ?
 enfant-f|Oui, une cabane.
 narrateur|Maman tend le coussin.
-narrateur|Il est moelleux.
+narrateur|Il est moelleux, un peu lourd.
 narrateur|Sarah veut le glisser dessous.
+narrateur|Elle pousse fort, d'un coup.
 narrateur|Une voiture touche son genou.
 enfant-f|Aïe.
 papa|La voiture est là.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Ses épaules tombent un peu.
 enfant-f|Où est mon doudou ?
 maman|Sur la chaise, peut-être ?
 narrateur|Sarah sort la tête.
@@ -1369,11 +1389,18 @@
 narrateur|Elle fouille le tissu.
 narrateur|Rien.
 enfant-f|Il est perdu.
-papa|Les voitures sont encore au sol.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes sous les voitures ?
 enfant-f|Je veux voir dessous.
 narrateur|Sarah prend une voiture bleue.
-narrateur|Elle la pose dans la caisse bleue.
+narrateur|Elle la pose dans la caisse.
 narrateur|Clac.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>torchon,cuillere,voitures</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1432,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah cherche son doudou. Où est-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah cherche son &lt;emphasis level="moderate"&gt;doudou&lt;/emphasis&gt;. Où est-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le jeu est fini. Que fait Kenza ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah cherche son &lt;emphasis&gt;doudou&lt;/emphasis&gt;. Où est-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1473,7 +1500,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1481,10 +1508,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1499,34 +1526,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>doudou</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1535,13 +1566,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1551,7 +1582,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_doudou_est_dessous; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1584,17 +1615,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Une deuxième voiture va dans la caisse. Clac. Tu regardes bien sous les roues ? Oui, maman. Un bout de tapis reparaît. Encore une, tout doux. Sarah glisse la troisième. Clac. Un coin de tissu rose. Mon doudou ! Le doudou était sous les voitures. Il sent encore le savon de la nappe. Sarah le serre contre sa joue. Le tissu est chaud, tout doux. Merci, tu l'as trouvé. Te voilà, petit. Il était dessous. La caisse bleue est presque pleine. Sous la table, le tapis est libre. L'ombre de la chaise reste là.</t>
+          <t>Une deuxième voiture va dans la caisse. Clac. Tu regardes bien sous les roues ? Oui, maman. Un bout de tapis reparaît. Sarah glisse la troisième. Clac. Un coin de tissu rose. Je le prends, d'un coup ! Elle tire trop fort. Les voitures retombent dessus. Oh. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sarah recule d'un pas. Je ne fonce pas. Elle refuse de tirer plus fort. Personne ne dit la réponse. Sarah observe les voitures, un instant. Sous le pied, l'éclat d'ombre brille. Il montre le doudou. Elle pose un genou au sol. Elle sort la dernière, sans se presser. Clac. Le tapis reparaît, rose au milieu. Mon doudou ! Le doudou était sous les voitures. Il sent le savon de la nappe. Sarah le serre contre sa joue. Le tissu est chaud, un peu plat. Merci, tu l'as trouvé. Te voilà, petit. Il était dessous. La caisse bleue est presque pleine. Sous la table, le tapis est libre. L'ombre de la chaise reste là.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Une deuxième voiture va dans la caisse. Clac. Tu regardes bien sous les roues ? Oui, maman. Un bout de tapis reparaît. Encore une, tout doux. Sarah glisse la troisième. Clac. Un coin de tissu rose. Mon doudou ! Le doudou était sous les voitures. Il sent encore le savon de la nappe. Sarah le serre contre sa joue. Le tissu est chaud, tout doux. Merci, tu l'as trouvé. Te voilà, petit. Il était dessous. La caisse bleue est presque pleine. Sous la table, le tapis est libre. L'ombre de la chaise reste là.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une deuxième voiture va dans la caisse. Clac. Tu regardes bien sous les roues ? Oui, maman. Un bout de tapis reparaît. Sarah glisse la troisième. Clac. Un coin de tissu rose. Je le prends, d'un coup ! Elle tire trop fort. Les voitures retombent dessus. Oh. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sarah recule d'un pas. Je ne fonce pas. Elle refuse de tirer plus fort. Personne ne dit la réponse. Sarah observe les voitures, un instant. Sous le pied, l'&lt;emphasis level="moderate"&gt;éclat d'ombre&lt;/emphasis&gt; brille. Il montre le doudou. Elle pose un genou au sol. Elle sort la dernière, sans se presser. Clac. Le tapis reparaît, rose au milieu. Mon doudou ! Le doudou était sous les voitures. Il sent le savon de la nappe. Sarah le serre contre sa joue. Le tissu est chaud, un peu plat. Merci, tu l'as trouvé. Te voilà, petit. Il était dessous. La caisse bleue est presque pleine. Sous la table, le tapis est libre. L'ombre de la chaise reste là.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Kenza a rangé. Les voitures sont dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Papa était là.&lt;/slow&gt; [pause]</t>
+          <t>Une deuxième voiture va dans la caisse. Clac. Tu regardes bien sous les roues ? Oui, maman. Un bout de tapis reparaît. Sarah glisse la troisième. Clac. Un coin de tissu rose. Je le prends, d'un coup ! Elle tire trop fort. Les voitures retombent dessus. Oh. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sarah recule d'un pas. Je ne fonce pas. Elle refuse de tirer plus fort. Personne ne dit la réponse. Sarah observe les voitures, un instant. Sous le pied, l'&lt;emphasis&gt;éclat d'ombre&lt;/emphasis&gt; brille. Il montre le doudou. Elle pose un genou au sol. Elle sort la dernière, sans se presser. Clac. Le tapis reparaît, rose au milieu. Mon doudou ! Le doudou était sous les voitures. Il sent le savon de la nappe. Sarah le serre contre sa joue. Le tissu est chaud, un peu plat. Merci, tu l'as trouvé. Te voilà, petit. Il était dessous. La caisse bleue est presque pleine. Sous la table, le tapis est libre. L'ombre de la chaise reste là. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1641,7 +1672,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1649,10 +1680,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1675,30 +1706,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>éclat d'ombre</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1707,10 +1738,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1719,11 +1750,11 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
@@ -1733,15 +1764,30 @@
 maman|Tu regardes bien sous les roues ?
 enfant-f|Oui, maman.
 narrateur|Un bout de tapis reparaît.
-papa|Encore une, tout doux.
 narrateur|Sarah glisse la troisième.
 narrateur|Clac.
 narrateur|Un coin de tissu rose.
+enfant-f|Je le prends, d'un coup !
+narrateur|Elle tire trop fort.
+narrateur|Les voitures retombent dessus.
+enfant-f|Oh.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Sarah recule d'un pas.
+enfant-f|Je ne fonce pas.
+narrateur|Elle refuse de tirer plus fort.
+narrateur|Personne ne dit la réponse.
+narrateur|Sarah observe les voitures, un instant.
+narrateur|Sous le pied, l'éclat d'ombre brille.
+enfant-f|Il montre le doudou.
+narrateur|Elle pose un genou au sol.
+narrateur|Elle sort la dernière, sans se presser.
+narrateur|Clac.
+narrateur|Le tapis reparaît, rose au milieu.
 enfant-f|Mon doudou !
 narrateur|Le doudou était sous les voitures.
-narrateur|Il sent encore le savon de la nappe.
+narrateur|Il sent le savon de la nappe.
 narrateur|Sarah le serre contre sa joue.
-narrateur|Le tissu est chaud, tout doux.
+narrateur|Le tissu est chaud, un peu plat.
 papa|Merci, tu l'as trouvé.
 maman|Te voilà, petit.
 enfant-f|Il était dessous.
@@ -1750,6 +1796,11 @@
 narrateur|L'ombre de la chaise reste là.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>caisse,voitures</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1774,17 +1825,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah glisse le coussin sous la table. Le coussin est moelleux. C'est ma cabane. Une cabane toute douce. Elle s'assoit, le doudou sur les genoux. La nappe fait un plafond. On frappe avant d'entrer ? Toc toc. On peut entrer ? Oui, papa. Papa se penche un peu. L'ombre est calme, maintenant. Tu veux un peu d'eau ? Oui, maman. Sarah boit une gorgée. Le doudou reste contre elle. Une ligne claire est encore au sol.</t>
+          <t>On met le coussin ? Sarah glisse le coussin sous la table. Le coussin est moelleux. C'est ma cabane. Une cabane pour toi. Elle s'assoit, le doudou sur les genoux. La nappe fait un plafond. On frappe avant d'entrer ? Toc toc. On peut entrer ? Oui, papa. Papa se penche un peu. L'ombre sent le savon. Tu veux un peu d'eau ? Oui, maman. Sarah boit une gorgée. L'eau est fraîche, un peu. Le doudou reste contre elle. Une ligne claire coupe le sol. On est bien, ici. Oui, très bien. Sarah pose la main sur la nappe. Le tissu est un peu humide. On entend la cuillère ? Elle est loin, maintenant. Sarah écoute. La maison est tranquille.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah glisse le coussin sous la table. Le coussin est moelleux. C'est ma cabane. Une cabane toute douce. Elle s'assoit, le doudou sur les genoux. La nappe fait un plafond. On frappe avant d'entrer ? Toc toc. On peut entrer ? Oui, papa. Papa se penche un peu. L'ombre est calme, maintenant. Tu veux un peu d'eau ? Oui, maman. Sarah boit une gorgée. Le doudou reste contre elle. Une ligne claire est encore au sol.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On met le coussin ? Sarah glisse le coussin sous la table. Le coussin est moelleux. C'est ma &lt;emphasis level="moderate"&gt;cabane&lt;/emphasis&gt;. Une cabane pour toi. Elle s'assoit, le doudou sur les genoux. La nappe fait un plafond. On frappe avant d'entrer ? Toc toc. On peut entrer ? Oui, papa. Papa se penche un peu. L'ombre sent le savon. Tu veux un peu d'eau ? Oui, maman. Sarah boit une gorgée. L'eau est fraîche, un peu. Le doudou reste contre elle. Une ligne claire coupe le sol. On est bien, ici. Oui, très bien. Sarah pose la main sur la nappe. Le tissu est un peu humide. On entend la cuillère ? Elle est loin, maintenant. Sarah écoute. La maison est tranquille.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Kenza se lave les mains. Papa range la &lt;emphasis&gt;caisse&lt;/emphasis&gt;.&lt;/slow&gt; [pause]</t>
+          <t>On met le coussin ? Sarah glisse le coussin sous la table. Le coussin est moelleux. C'est ma &lt;emphasis&gt;cabane&lt;/emphasis&gt;. Une cabane pour toi. Elle s'assoit, le doudou sur les genoux. La nappe fait un plafond. On frappe avant d'entrer ? Toc toc. On peut entrer ? Oui, papa. Papa se penche un peu. L'ombre sent le savon. Tu veux un peu d'eau ? Oui, maman. Sarah boit une gorgée. L'eau est fraîche, un peu. Le doudou reste contre elle. Une ligne claire coupe le sol. On est bien, ici. Oui, très bien. Sarah pose la main sur la nappe. Le tissu est un peu humide. On entend la cuillère ? Elle est loin, maintenant. Sarah écoute. La maison est tranquille. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1831,7 +1882,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1839,10 +1890,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1865,30 +1916,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>cabane</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1897,10 +1948,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1909,15 +1960,20 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=la_cabane_prend_place; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah glisse le coussin sous la table.
+          <t>papa|On met le coussin ?
+narrateur|Sarah glisse le coussin sous la table.
 narrateur|Le coussin est moelleux.
 enfant-f|C'est ma cabane.
-maman|Une cabane toute douce.
+maman|Une cabane pour toi.
 narrateur|Elle s'assoit, le doudou sur les genoux.
 narrateur|La nappe fait un plafond.
 papa|On frappe avant d'entrer ?
@@ -1925,12 +1981,26 @@
 papa|On peut entrer ?
 enfant-f|Oui, papa.
 narrateur|Papa se penche un peu.
-narrateur|L'ombre est calme, maintenant.
+narrateur|L'ombre sent le savon.
 maman|Tu veux un peu d'eau ?
 enfant-f|Oui, maman.
 narrateur|Sarah boit une gorgée.
+narrateur|L'eau est fraîche, un peu.
 narrateur|Le doudou reste contre elle.
-narrateur|Une ligne claire est encore au sol.</t>
+narrateur|Une ligne claire coupe le sol.
+enfant-f|On est bien, ici.
+papa|Oui, très bien.
+narrateur|Sarah pose la main sur la nappe.
+narrateur|Le tissu est un peu humide.
+enfant-f|On entend la cuillère ?
+papa|Elle est loin, maintenant.
+narrateur|Sarah écoute.
+narrateur|La maison est tranquille.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>coussin,toc</t>
         </is>
       </c>
     </row>
@@ -1957,17 +2027,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou est dans la cabane. Toi aussi. Bravo, tu l'as retrouvé. La nappe sent encore le savon. L'ombre de la chaise est douce, maintenant.</t>
+          <t>Le doudou est dans la cabane. Toi aussi. Tu le serres bien ? Oui, papa. La nappe sent le savon. Au plafond, un éclat d'ombre brille. Comme au pied de la chaise ! Tu le vois, toi ? Oui, il est là. Sarah le montre du doigt. Ma cabane est prête. Elle te va bien. Le savon reste dans l'air. L'éclat d'ombre dore la nappe.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou est dans la cabane. Toi aussi. Bravo, tu l'as retrouvé. La nappe sent encore le savon. L'ombre de la chaise est douce, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou est dans la cabane. Toi aussi. Tu le serres bien ? Oui, papa. La nappe sent le savon. Au plafond, un &lt;emphasis level="moderate"&gt;éclat d'ombre&lt;/emphasis&gt; brille. Comme au pied de la chaise ! Tu le vois, toi ? Oui, il est là. Sarah le montre du doigt. Ma cabane est prête. Elle te va bien. Le savon reste dans l'air. L'éclat d'ombre dore la nappe.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou est dans la cabane. Toi aussi. Tu le serres bien ? Oui, papa. La nappe sent le savon. Au plafond, un &lt;emphasis&gt;éclat d'ombre&lt;/emphasis&gt; brille. Comme au pied de la chaise ! Tu le vois, toi ? Oui, il est là. Sarah le montre du doigt. Ma cabane est prête. Elle te va bien. Le savon reste dans l'air. L'éclat d'ombre dore la nappe.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2014,18 +2084,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2034,12 +2104,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2048,17 +2118,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'ombre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2067,11 +2141,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2080,28 +2154,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_éclat_du_pied_dore_la_nappe; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>enfant-f|Le doudou est dans la cabane.
 maman|Toi aussi.
-papa|Bravo, tu l'as retrouvé.
-narrateur|La nappe sent encore le savon.
-narrateur|L'ombre de la chaise est douce, maintenant.</t>
+papa|Tu le serres bien ?
+enfant-f|Oui, papa.
+narrateur|La nappe sent le savon.
+narrateur|Au plafond, un éclat d'ombre brille.
+enfant-f|Comme au pied de la chaise !
+papa|Tu le vois, toi ?
+enfant-f|Oui, il est là.
+narrateur|Sarah le montre du doigt.
+enfant-f|Ma cabane est prête.
+maman|Elle te va bien.
+narrateur|Le savon reste dans l'air.
+narrateur|L'éclat d'ombre dore la nappe.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>nappe</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2214,6 +2306,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>